<commit_message>
Switch from Google Form to Apps Script web app (auto write/read of the shared sheet)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M3YQQoTMjJVd24svSbk5Ra
</commit_message>
<xml_diff>
--- a/ATI_Monitor_Shared_TEMPLATE.xlsx
+++ b/ATI_Monitor_Shared_TEMPLATE.xlsx
@@ -582,21 +582,21 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2. Share &gt; "Anyone with the link" = Editor. Copy the link (the sharing link). / 共有 ▸「リンクを知っている全員」を「編集者」に。リンク(共有リンク)をコピー。</t>
+          <t>2. In the sheet: Extensions &gt; Apps Script. Delete the sample code, paste the script (the app: Share &gt; Google Sheet connection &gt; Copy script) and save. / シートで「拡張機能 ▸ Apps Script」。サンプルのコードを消し、スクリプトを貼って保存(アプリの Share ▸ Google Sheet connection ▸ Copy script でコピーできる)。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>3. File &gt; Share &gt; Publish to web &gt; Link: choose the sheet "Data" (not Entire document), format CSV &gt; Publish. Copy the link (the compare link). / 「ファイル ▸ 共有 ▸ ウェブに公開」▸ リンク: シート「Data」を選び、形式CSVで公開。リンク(比較用リンク)をコピー。</t>
+          <t>3. Deploy &gt; New deployment &gt; type: Web app. Execute as: Me. Who has access: Anyone. Press Deploy, authorize, and copy the web app URL. / 「デプロイ ▸ 新しいデプロイ」▸ 種類「ウェブアプリ」。次のユーザーとして実行: 自分。アクセスできるユーザー: 全員。デプロイして承認し、ウェブアプリのURLをコピー。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>4. Give students: the app address, the sharing link, the compare link. / 学生に、アプリのアドレス・共有リンク・比較用リンクを伝える。</t>
+          <t>4. In the app: Share &gt; Google Sheet connection: paste the URL, press "Test connection", then "Create class setup link". Send that link to the students. / アプリの Share ▸ Google Sheet connection に URL を貼り、「Test connection」▸「Create class setup link」。できたリンクを学生に送る。</t>
         </is>
       </c>
     </row>
@@ -613,45 +613,45 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>In the app: Share &gt; Copy my data. Open this sheet, tab "Data", click the first empty cell of column A (below the last row) and paste. / アプリの Share ▸「Copy my data」。このシートの「Data」タブで、A列の最初の空のセル(最終行の下)をクリックして貼り付ける。</t>
+          <t>Open the class setup link once. After that the app writes your data into this sheet automatically each time you save. Nothing is pasted by hand. / クラス設定リンクを1回開く。あとは、保存のたびに、アプリが自動でこのシートに書き込む。手で貼り付ける必要はない。</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Paste again after every correction. Only the newest paste of each ATI is used. / 直したら、もう一度貼る。ATIごとに最も新しい貼り付けだけが使われる。</t>
-        </is>
-      </c>
+      <c r="A11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr"/>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Rules / 決まり</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Rules / 決まり</t>
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Do not change the header rows or the tab names (Data, ATIs, _Store). / 見出し行とタブ名(Data、ATIs、_Store)は変えない。</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Do not change the header row, the order of the columns, or the sheet name "Data". / 見出し行・列の順序・シート名「Data」は変えない。</t>
+          <t>The tabs are filled in by the script. Do not type into them; the app replaces the rows of an ATI on every save. / タブはスクリプトが書く。手で入力しない。保存のたびに、アプリがそのATIの行を置き換える。</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Column B "Upload" is filled in by the app (date and time of the paste). Old pastes may be deleted by the administrator. / 列B「Upload」はアプリが入れる(貼り付けの日時)。古い貼り付けは、管理者が消してよい。</t>
+          <t>Data = readable daily results (Type: Info, WL, Tiller, Fertilizer, Pesticide). ATIs = one summary row per ATI. _Store = hidden machine copy used by the app. / Data=読める毎日の結果。ATIs=ATIごとの要約。_Store=アプリが使う隠しタブ。</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Type: Info (place, sowing date), WL (daily water level and irrigation), Tiller, Fertilizer, Pesticide. / Type: Info(場所・播種日)、WL(毎日の水位と灌漑)、Tiller、Fertilizer、Pesticide。</t>
+          <t>Menu "ATI Monitor" in the sheet: Show web app URL, Check sheets, Delete ALL ATI data. / シートのメニュー「ATI Monitor」: Show web app URL、Check sheets、Delete ALL ATI data。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rename ATI to Site, teacher to administrator, students to users; app name 3F4D Water Monitor
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M3YQQoTMjJVd24svSbk5Ra
</commit_message>
<xml_diff>
--- a/ATI_Monitor_Shared_TEMPLATE.xlsx
+++ b/ATI_Monitor_Shared_TEMPLATE.xlsx
@@ -464,7 +464,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ATI</t>
+          <t>Site</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -558,7 +558,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>ATI Monitor shared sheet (template) / 共有シート(雛形)</t>
+          <t>Site Monitor shared sheet (template) / 共有シート(雛形)</t>
         </is>
       </c>
     </row>
@@ -596,7 +596,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>4. In the app: Share &gt; Google Sheet connection: paste the URL, press "Test connection", then "Create class setup link". Send that link to the students. / アプリの Share ▸ Google Sheet connection に URL を貼り、「Test connection」▸「Create class setup link」。できたリンクを学生に送る。</t>
+          <t>4. In the app: Share &gt; Google Sheet connection: paste the URL, press "Test connection", then "Create class setup link". Send that link to the users. / アプリの Share ▸ Google Sheet connection に URL を貼り、「Test connection」▸「Create class setup link」。できたリンクを利用者に送る。</t>
         </is>
       </c>
     </row>
@@ -606,7 +606,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>For students / 学生の使い方</t>
+          <t>For users / 利用者の使い方</t>
         </is>
       </c>
     </row>
@@ -630,28 +630,28 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Do not change the header rows or the tab names (Data, ATIs, _Store). / 見出し行とタブ名(Data、ATIs、_Store)は変えない。</t>
+          <t>Do not change the header rows or the tab names (Data, sites, _Store). / 見出し行とタブ名(Data、sites、_Store)は変えない。</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>The tabs are filled in by the script. Do not type into them; the app replaces the rows of an ATI on every save. / タブはスクリプトが書く。手で入力しない。保存のたびに、アプリがそのATIの行を置き換える。</t>
+          <t>The tabs are filled in by the script. Do not type into them; the app replaces the rows of an site on every save. / タブはスクリプトが書く。手で入力しない。保存のたびに、アプリがそのサイトの行を置き換える。</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Data = readable daily results (Type: Info, WL, Tiller, Fertilizer, Pesticide). ATIs = one summary row per ATI. _Store = hidden machine copy used by the app. / Data=読める毎日の結果。ATIs=ATIごとの要約。_Store=アプリが使う隠しタブ。</t>
+          <t>Data = readable daily results (Type: Info, WL, Tiller, Fertilizer, Pesticide). Sites = one summary row per site. _Store = hidden machine copy used by the app. / Data=読める毎日の結果。sites=サイトごとの要約。_Store=アプリが使う隠しタブ。</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Menu "ATI Monitor" in the sheet: Show web app URL, Check sheets, Delete ALL ATI data. / シートのメニュー「ATI Monitor」: Show web app URL、Check sheets、Delete ALL ATI data。</t>
+          <t>Menu "Site Monitor" in the sheet: Show web app URL, Check sheets, Delete ALL site data. / シートのメニュー「site Monitor」: Show web app URL、Check sheets、Delete ALL site data。</t>
         </is>
       </c>
     </row>

</xml_diff>